<commit_message>
Reset cloud baseline to run 2026-10-13_183310
header_compare.py now excludes the Sitecore context nav (b9efbcd). The
previous baseline (2026-10-09_133040) predates that change, so every
nightly run reported the context-nav links as removed (16 header locales
shown as Improved). The new baseline was captured with the current
script; the old one stays in history at 1aa69a2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/baselines/cloud_baseline/FooterCheck_Report.xlsx
+++ b/baselines/cloud_baseline/FooterCheck_Report.xlsx
@@ -2319,7 +2319,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Cookie Settings (/en/global/company/press/2026/teamviewer-expands-ai-powered-it-troubleshooting-from-guidance-to-governed-action) | Existing Partner Login (/en/partner/existing-partner-login)</t>
+          <t>Cookies Settings (/en/global/company/press/2026/teamviewer-expands-ai-powered-it-troubleshooting-from-guidance-to-governed-action) | Existing Partner Login (/en/partner/existing-partner-login)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -31771,7 +31771,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Cookie Settings</t>
+          <t>Cookies Settings</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">

</xml_diff>